<commit_message>
Architecture Supabase Cloud complète : Persistance temps réel pour Événements, Produits Boutique, Articles Gazette, Émargement Foyer QR et Logs Audit
</commit_message>
<xml_diff>
--- a/public/data/Registre_Officiel_Adherents_Cotisations_2026-2027.xlsx
+++ b/public/data/Registre_Officiel_Adherents_Cotisations_2026-2027.xlsx
@@ -398,27 +398,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
     <col min="3" max="3" width="32.83203125" customWidth="1"/>
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="34.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="38.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
     <col min="9" max="9" width="34.83203125" customWidth="1"/>
-    <col min="10" max="10" width="24.83203125" customWidth="1"/>
-    <col min="11" max="11" width="26.83203125" customWidth="1"/>
-    <col min="12" max="12" width="34.83203125" customWidth="1"/>
-    <col min="13" max="13" width="55.83203125" customWidth="1"/>
-    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="24.83203125" customWidth="1"/>
+    <col min="12" max="12" width="45.83203125" customWidth="1"/>
+    <col min="13" max="13" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Matricule Adhérent</v>
+        <v>Matricule Officiel</v>
       </c>
       <c r="B1" t="str">
         <v>Nom &amp; Prénom</v>
@@ -427,404 +426,213 @@
         <v>Email Étudiant</v>
       </c>
       <c r="D1" t="str">
-        <v>Promotion / Année</v>
+        <v>Promotion / Filière</v>
       </c>
       <c r="E1" t="str">
-        <v>Rôle Associatif</v>
+        <v>Rôle Plateforme</v>
       </c>
       <c r="F1" t="str">
-        <v>État du Compte</v>
+        <v>Statut Cotisation (10€)</v>
       </c>
       <c r="G1" t="str">
-        <v>Statut Cotisation</v>
+        <v>Montant Encaissé</v>
       </c>
       <c r="H1" t="str">
-        <v>Montant Cotisation</v>
+        <v>Date Validation</v>
       </c>
       <c r="I1" t="str">
-        <v>Moyen de Règlement</v>
+        <v>Mode de Paiement</v>
       </c>
       <c r="J1" t="str">
-        <v>Date de Validation / Création</v>
+        <v>Date Expiration Pass</v>
       </c>
       <c r="K1" t="str">
-        <v>Validé / Modifié Par</v>
+        <v>Code Unique Contrôle</v>
       </c>
       <c r="L1" t="str">
-        <v>Code Sécurité QR</v>
+        <v>URL Contrôle Guichetier</v>
       </c>
       <c r="M1" t="str">
-        <v>Lien Contrôle QR Code</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Date d'Expiration</v>
+        <v>Terroirs Favoris</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ECE-TERR-2026-2883</v>
+        <v>ECE-TERR-2026-3131</v>
       </c>
       <c r="B2" t="str">
-        <v>Jules Houry</v>
+        <v>Arthur Rimbaud</v>
       </c>
       <c r="C2" t="str">
-        <v>jules.houry@edu.ece.fr</v>
+        <v>arthur.rimbaud@edu.ece.fr</v>
       </c>
       <c r="D2" t="str">
-        <v>Ingé 4 (Promo 2028)</v>
+        <v>ING1 (Promo 2029)</v>
       </c>
       <c r="E2" t="str">
-        <v>🛡️ Bureau Exécutif</v>
+        <v>Visiteur</v>
       </c>
       <c r="F2" t="str">
-        <v>🟢 Actif</v>
+        <v>⚪ Non Adhérent (Visiteur)</v>
       </c>
       <c r="G2" t="str">
-        <v>✅ Validée &amp; Active (Bureau Fondateur)</v>
+        <v>0,00 €</v>
       </c>
       <c r="H2" t="str">
-        <v>10,00 € (Inclus Bureau)</v>
+        <v>N/A</v>
       </c>
       <c r="I2" t="str">
-        <v>Exonéré (Bureau Fondateur)</v>
+        <v>Aucun (Non adhérent)</v>
       </c>
       <c r="J2" t="str">
-        <v>10 janv. 2026, 11:00</v>
+        <v>N/A</v>
       </c>
       <c r="K2" t="str">
-        <v>Jules Houry (Président)</v>
+        <v>QR-AUTH-3131-ECE-TERROIR-2026-VALIDE</v>
       </c>
       <c r="L2" t="str">
-        <v>QR-AUTH-2883-ECE-TERROIR-2026-VALIDE</v>
+        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-3131</v>
       </c>
       <c r="M2" t="str">
-        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-2883</v>
-      </c>
-      <c r="N2" t="str">
-        <v>31/08/2027</v>
+        <v>Ardennes, Bourgogne</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ECE-TERR-2026-2683</v>
+        <v>ECE-TERR-2026-2883</v>
       </c>
       <c r="B3" t="str">
-        <v>Thomas Petit</v>
+        <v>Jules Houry</v>
       </c>
       <c r="C3" t="str">
-        <v>thomas.petit@edu.ece.fr</v>
+        <v>jules.houry@edu.ece.fr</v>
       </c>
       <c r="D3" t="str">
-        <v>Ingé 4 (Promo 2028)</v>
+        <v>Visiteur ECE</v>
       </c>
       <c r="E3" t="str">
-        <v>🛡️ Bureau Exécutif</v>
+        <v>Administrateur Bureau</v>
       </c>
       <c r="F3" t="str">
-        <v>🟢 Actif</v>
+        <v>✅ Validée &amp; Active (Bureau Fondateur)</v>
       </c>
       <c r="G3" t="str">
-        <v>✅ Validée &amp; Active (Bureau Fondateur)</v>
+        <v>10,00 € (Inclus Bureau)</v>
       </c>
       <c r="H3" t="str">
-        <v>10,00 € (Inclus Bureau)</v>
+        <v>Adhésion Initiale 2026</v>
       </c>
       <c r="I3" t="str">
         <v>Exonéré (Bureau Fondateur)</v>
       </c>
       <c r="J3" t="str">
-        <v>12 janv. 2026, 12:30</v>
+        <v>31/08/2027</v>
       </c>
       <c r="K3" t="str">
-        <v>Jules Houry (Président)</v>
+        <v>QR-AUTH-2883-ECE-TERROIR-2026-VALIDE</v>
       </c>
       <c r="L3" t="str">
-        <v>QR-AUTH-2683-ECE-TERROIR-2026-VALIDE</v>
+        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-2883</v>
       </c>
       <c r="M3" t="str">
-        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-2683</v>
-      </c>
-      <c r="N3" t="str">
-        <v>31/08/2027</v>
+        <v>Savoie, Bourgogne, Jura</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ECE-TERR-2026-1124</v>
+        <v>ECE-TERR-2026-2683</v>
       </c>
       <c r="B4" t="str">
-        <v>Léonard Brault</v>
+        <v>Thomas Petit</v>
       </c>
       <c r="C4" t="str">
-        <v>leonard.brault@edu.ece.fr</v>
+        <v>thomas.petit@edu.ece.fr</v>
       </c>
       <c r="D4" t="str">
-        <v>Ingé 4 (Promo 2028)</v>
+        <v>ING4 (Promo 2028)</v>
       </c>
       <c r="E4" t="str">
-        <v>🍷 Membre Adhérent</v>
+        <v>Administrateur Bureau</v>
       </c>
       <c r="F4" t="str">
-        <v>🟢 Actif</v>
+        <v>✅ Validée &amp; Active (Bureau Fondateur)</v>
       </c>
       <c r="G4" t="str">
-        <v>✅ Validée &amp; Active (2026-2027)</v>
+        <v>10,00 € (Inclus Bureau)</v>
       </c>
       <c r="H4" t="str">
-        <v>10,00 €</v>
+        <v>Adhésion Initiale 2026</v>
       </c>
       <c r="I4" t="str">
-        <v>HelloAsso / En ligne</v>
+        <v>Exonéré (Bureau Fondateur)</v>
       </c>
       <c r="J4" t="str">
-        <v>1 févr. 2026, 15:00</v>
+        <v>31/08/2027</v>
       </c>
       <c r="K4" t="str">
-        <v>Bureau ECE Terroir</v>
+        <v>QR-AUTH-2683-ECE-TERROIR-2026-VALIDE</v>
       </c>
       <c r="L4" t="str">
-        <v>QR-AUTH-1124-ECE-TERROIR-2026-VALIDE</v>
+        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-2683</v>
       </c>
       <c r="M4" t="str">
-        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-1124</v>
-      </c>
-      <c r="N4" t="str">
-        <v>31/08/2027</v>
+        <v>Savoie, Bourgogne, Jura</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ECE-TERR-2026-3952</v>
+        <v>ECE-TERR-2026-1124</v>
       </c>
       <c r="B5" t="str">
-        <v>Jerry Wang</v>
+        <v>Léonard Brault</v>
       </c>
       <c r="C5" t="str">
-        <v>jerry.wang@edu.ece.fr</v>
+        <v>leonard.brault@edu.ece.fr</v>
       </c>
       <c r="D5" t="str">
-        <v>Ingé 4 (Promo 2028)</v>
+        <v>ING4 (Promo 2028)</v>
       </c>
       <c r="E5" t="str">
-        <v>🛡️ Bureau Exécutif</v>
+        <v>Administrateur Bureau</v>
       </c>
       <c r="F5" t="str">
-        <v>🟢 Actif</v>
+        <v>✅ Validée &amp; Active (Bureau Fondateur)</v>
       </c>
       <c r="G5" t="str">
-        <v>✅ Validée &amp; Active (Bureau Fondateur)</v>
+        <v>10,00 € (Inclus Bureau)</v>
       </c>
       <c r="H5" t="str">
-        <v>10,00 € (Inclus Bureau)</v>
+        <v>Adhésion Initiale 2026</v>
       </c>
       <c r="I5" t="str">
         <v>Exonéré (Bureau Fondateur)</v>
       </c>
       <c r="J5" t="str">
-        <v>15 janv. 2026, 10:00</v>
+        <v>31/08/2027</v>
       </c>
       <c r="K5" t="str">
-        <v>Jules Houry (Président)</v>
+        <v>QR-AUTH-1124-ECE-TERROIR-2026-VALIDE</v>
       </c>
       <c r="L5" t="str">
-        <v>QR-AUTH-3952-ECE-TERROIR-2026-VALIDE</v>
+        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-1124</v>
       </c>
       <c r="M5" t="str">
-        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-3952</v>
-      </c>
-      <c r="N5" t="str">
-        <v>31/08/2027</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>ECE-TERR-2026-4471</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Emma Roy</v>
-      </c>
-      <c r="C6" t="str">
-        <v>emma.roy@edu.ece.fr</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Ingé 1 (Promo 2029)</v>
-      </c>
-      <c r="E6" t="str">
-        <v>🍷 Membre Adhérent</v>
-      </c>
-      <c r="F6" t="str">
-        <v>🟢 Actif</v>
-      </c>
-      <c r="G6" t="str">
-        <v>✅ Validée &amp; Active (2026-2027)</v>
-      </c>
-      <c r="H6" t="str">
-        <v>10,00 €</v>
-      </c>
-      <c r="I6" t="str">
-        <v>HelloAsso / En ligne</v>
-      </c>
-      <c r="J6" t="str">
-        <v>15 août 2026, 18:20</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Bureau ECE Terroir</v>
-      </c>
-      <c r="L6" t="str">
-        <v>QR-AUTH-4471-ECE-TERROIR-2026-VALIDE</v>
-      </c>
-      <c r="M6" t="str">
-        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-4471</v>
-      </c>
-      <c r="N6" t="str">
-        <v>31/08/2027</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>ECE-TERR-2026-3323</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Antoine Dubois</v>
-      </c>
-      <c r="C7" t="str">
-        <v>antoine.dubois@edu.ece.fr</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Mastère (Promo 2026)</v>
-      </c>
-      <c r="E7" t="str">
-        <v>🍷 Membre Adhérent</v>
-      </c>
-      <c r="F7" t="str">
-        <v>🟢 Actif</v>
-      </c>
-      <c r="G7" t="str">
-        <v>✅ Validée &amp; Active (2026-2027)</v>
-      </c>
-      <c r="H7" t="str">
-        <v>10,00 €</v>
-      </c>
-      <c r="I7" t="str">
-        <v>HelloAsso / En ligne</v>
-      </c>
-      <c r="J7" t="str">
-        <v>20 août 2026, 12:00</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Bureau ECE Terroir</v>
-      </c>
-      <c r="L7" t="str">
-        <v>QR-AUTH-3323-ECE-TERROIR-2026-VALIDE</v>
-      </c>
-      <c r="M7" t="str">
-        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-3323</v>
-      </c>
-      <c r="N7" t="str">
-        <v>31/08/2027</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>ECE-TERR-2026-4981</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Maxime Lefebvre</v>
-      </c>
-      <c r="C8" t="str">
-        <v>maxime.lefebvre@edu.ece.fr</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Ingé 2 (Promo 2028)</v>
-      </c>
-      <c r="E8" t="str">
-        <v>👤 Visiteur Non-Adhérent</v>
-      </c>
-      <c r="F8" t="str">
-        <v>🟢 Actif</v>
-      </c>
-      <c r="G8" t="str">
-        <v>⏳ En attente de validation / paiement</v>
-      </c>
-      <c r="H8" t="str">
-        <v>10,00 € (En attente)</v>
-      </c>
-      <c r="I8" t="str">
-        <v>Carte Bancaire / HelloAsso</v>
-      </c>
-      <c r="J8" t="str">
-        <v>25 août 2026, 16:25</v>
-      </c>
-      <c r="K8" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="L8" t="str">
-        <v>QR-AUTH-4981-ECE-TERROIR-2026-VALIDE</v>
-      </c>
-      <c r="M8" t="str">
-        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-4981</v>
-      </c>
-      <c r="N8" t="str">
-        <v>En cours</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>ECE-TERR-2026-4007</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Chloé Moreau</v>
-      </c>
-      <c r="C9" t="str">
-        <v>chloe.moreau@edu.ece.fr</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Ingé 1 (Promo 2029)</v>
-      </c>
-      <c r="E9" t="str">
-        <v>👤 Visiteur Non-Adhérent</v>
-      </c>
-      <c r="F9" t="str">
-        <v>🟢 Actif</v>
-      </c>
-      <c r="G9" t="str">
-        <v>⚪ Non Adhérent (Visiteur)</v>
-      </c>
-      <c r="H9" t="str">
-        <v>0,00 €</v>
-      </c>
-      <c r="I9" t="str">
-        <v>Espèces / Lydia au Foyer des Élèves</v>
-      </c>
-      <c r="J9" t="str">
-        <v>25 août 2026, 18:00</v>
-      </c>
-      <c r="K9" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="L9" t="str">
-        <v>QR-AUTH-4007-ECE-TERROIR-2026-VALIDE</v>
-      </c>
-      <c r="M9" t="str">
-        <v>http://localhost:3000/verifier?id=ECE-TERR-2026-4007</v>
-      </c>
-      <c r="N9" t="str">
-        <v>N/A</v>
+        <v>Savoie, Bourgogne, Jura</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C9"/>
   <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="45.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
     <col min="3" max="3" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -836,51 +644,51 @@
         <v>Valeur</v>
       </c>
       <c r="C1" t="str">
-        <v>Détail</v>
+        <v>Notes &amp; Détails</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Total Utilisateurs Enregistrés</v>
-      </c>
-      <c r="B2">
-        <v>8</v>
+        <v>Année Universitaire</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-2027</v>
       </c>
       <c r="C2" t="str">
-        <v>Totalité des comptes dans la base</v>
+        <v>Exercice en cours</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Adhérents Actifs &amp; Conformes (2026-2027)</v>
+        <v>Total Utilisateurs Enregistrés</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C3" t="str">
-        <v>Membres avec accès aux tarifs réduits</v>
+        <v>Comptes actifs sur la plateforme</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Membres du Bureau Exécutif</v>
+        <v>Nombre d'Adhérents Officiels (Pass Épicurien Actif)</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="str">
-        <v>Accès administrateurs actifs</v>
+        <v>Membres en règle de cotisation</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Visiteurs Non-Adhérents</v>
+        <v>Demandes d'Adhésion en Attente</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C5" t="str">
-        <v>Comptes créés sans cotisation validée</v>
+        <v>À vérifier et valider par le Bureau</v>
       </c>
     </row>
     <row r="6">
@@ -891,67 +699,45 @@
         <v>0</v>
       </c>
       <c r="C6" t="str">
-        <v>Comptes temporairement bloqués par le bureau</v>
+        <v>Accès aux avantages suspendu</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Total Cotisations Actives Encaissées (€)</v>
+        <v>Tarif Unitaire Cotisation</v>
       </c>
       <c r="B7" t="str">
-        <v>60,00 €</v>
+        <v>10,00 €</v>
       </c>
       <c r="C7" t="str">
-        <v>Cotisation officielle fixée à 10 € / an</v>
+        <v>Pass annuel donnant accès à -15% boutique et soirées</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Paiements HelloAsso (CB)</v>
-      </c>
-      <c r="B8">
-        <v>0</v>
+        <v>Total Cotisations Encaissées (TTC)</v>
+      </c>
+      <c r="B8" t="str">
+        <v>30,00 €</v>
       </c>
       <c r="C8" t="str">
-        <v>Directement versé sur compte bancaire ECE Terroir</v>
+        <v>Budget d'exploitation alloué aux festins et matériel</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Paiements Espèces au Foyer</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
+        <v>Dernière Synchronisation</v>
+      </c>
+      <c r="B9" t="str">
+        <v>30/08/2026 22:24:55</v>
       </c>
       <c r="C9" t="str">
-        <v>Caisse physique du Pôle Trésorerie</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Paiements Virement / Lydia</v>
-      </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Virements reçus</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Dernière Synchronisation Drive</v>
-      </c>
-      <c r="B11" t="str">
-        <v>26/08/2026 11:43:26</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Mise à jour automatique par la plateforme web</v>
+        <v>Généré automatiquement par la plateforme</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>